<commit_message>
FIX: Bakım JSON fallback kaldır - sadece proje-spesifik veri kullan, tüm projeler için maintenance.json oluştur
</commit_message>
<xml_diff>
--- a/data/iasi/Veriler.xlsx
+++ b/data/iasi/Veriler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\iasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DCFA36-B5D1-4D08-A44F-03F512E7981E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D77C5560-20FA-428C-A42B-A4AE6733100B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -863,7 +863,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2346,7 +2346,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
@@ -2380,7 +2380,7 @@
     </row>
     <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
-        <v>2219</v>
+        <v>2217</v>
       </c>
       <c r="B2" t="s">
         <v>198</v>
@@ -2403,7 +2403,7 @@
     </row>
     <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
-        <v>2220</v>
+        <v>2218</v>
       </c>
       <c r="B3" t="s">
         <v>186</v>
@@ -2423,7 +2423,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
-        <v>2221</v>
+        <v>2219</v>
       </c>
       <c r="C4" t="s">
         <v>191</v>
@@ -2440,7 +2440,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
-        <v>2222</v>
+        <v>2220</v>
       </c>
       <c r="C5" t="s">
         <v>195</v>
@@ -2451,7 +2451,7 @@
     </row>
     <row r="6" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>2223</v>
+        <v>2221</v>
       </c>
       <c r="C6" t="s">
         <v>197</v>
@@ -2459,122 +2459,147 @@
     </row>
     <row r="7" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
-        <v>2224</v>
+        <v>2222</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
-        <v>2225</v>
+        <v>2223</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
-        <v>2226</v>
+        <v>2224</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
-        <v>2227</v>
+        <v>2225</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
-        <v>2228</v>
+        <v>2226</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
-        <v>2229</v>
+        <v>2227</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
-        <v>2230</v>
+        <v>2228</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
-        <v>2231</v>
+        <v>2229</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
-        <v>2232</v>
+        <v>2230</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
-        <v>2233</v>
+        <v>2231</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
-        <v>2234</v>
+        <v>2232</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
-        <v>2235</v>
+        <v>2233</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
-        <v>2236</v>
+        <v>2234</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
-        <v>2237</v>
+        <v>2235</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
-        <v>2238</v>
+        <v>2236</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
-        <v>2239</v>
+        <v>2237</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
-        <v>2240</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
-        <v>2241</v>
+        <v>2239</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
-        <v>2242</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
-        <v>2243</v>
+        <v>2241</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
-        <v>2244</v>
+        <v>2242</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
-        <v>2245</v>
+        <v>2243</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
         <v>2246</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A30" s="18">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
         <v>2247</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33" s="18">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34" s="18">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35" s="18">
+        <v>2250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FIX: 2251 test aracını database'den sil (Excel'de yok)
</commit_message>
<xml_diff>
--- a/data/iasi/Veriler.xlsx
+++ b/data/iasi/Veriler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fatiherkin\Desktop\bozankaya_ssh_takip\data\iasi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D77C5560-20FA-428C-A42B-A4AE6733100B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99E13962-D642-4692-BEB1-295A02EC9C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -863,7 +863,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2346,7 +2346,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="23.33203125" bestFit="1" customWidth="1"/>
@@ -2602,6 +2602,9 @@
         <v>2250</v>
       </c>
     </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36" s="18"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>